<commit_message>
Clarify worksheet names and update layout notes
</commit_message>
<xml_diff>
--- a/Studymaterials/生活記録表生徒用_縦型.xlsx
+++ b/Studymaterials/生活記録表生徒用_縦型.xlsx
@@ -8,17 +8,17 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\nakag\Desktop\GitHub\Myownproject\Studymaterials\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{448A5ACA-6A2A-40AE-B89D-BA53BC044819}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{768ADFC3-A792-4567-8124-BDD40A62E4B9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="縦型1" sheetId="1" r:id="rId1"/>
-    <sheet name="縦型2" sheetId="2" r:id="rId2"/>
+    <sheet name="縦型日曜始まり" sheetId="1" r:id="rId1"/>
+    <sheet name="縦型月曜始まり" sheetId="2" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">縦型1!$A$1:$H$61</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="1">縦型2!$A$1:$H$61</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="1">縦型月曜始まり!$A$1:$H$61</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">縦型日曜始まり!$A$1:$H$61</definedName>
   </definedNames>
   <calcPr calcId="0"/>
 </workbook>

</xml_diff>